<commit_message>
Added a review flag to the prompt
</commit_message>
<xml_diff>
--- a/analysis/automatic_alternate_abbreviation_annotation/output/subset_alt_abbrev_annotation_manually_annotated_df.xlsx
+++ b/analysis/automatic_alternate_abbreviation_annotation/output/subset_alt_abbrev_annotation_manually_annotated_df.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="584">
   <si>
     <t>HGNC_ID</t>
   </si>
@@ -515,6 +515,1257 @@
   </si>
   <si>
     <t>mesenteric estrogen dependent adipogenesis</t>
+  </si>
+  <si>
+    <t>HGNC:13302</t>
+  </si>
+  <si>
+    <t>ENSG00000112218</t>
+  </si>
+  <si>
+    <t>GENE ID:81491</t>
+  </si>
+  <si>
+    <t>GPR63</t>
+  </si>
+  <si>
+    <t>PSP24(beta)</t>
+  </si>
+  <si>
+    <t>G protein-coupled receptor 63</t>
+  </si>
+  <si>
+    <t>HGNC:4055</t>
+  </si>
+  <si>
+    <t>ENSG00000196419</t>
+  </si>
+  <si>
+    <t>GENE ID:2547</t>
+  </si>
+  <si>
+    <t>XRCC6</t>
+  </si>
+  <si>
+    <t>D22S671</t>
+  </si>
+  <si>
+    <t>X-ray repair cross complementing 6</t>
+  </si>
+  <si>
+    <t>HGNC:12953</t>
+  </si>
+  <si>
+    <t>ENSG00000197279</t>
+  </si>
+  <si>
+    <t>GENE ID:7718</t>
+  </si>
+  <si>
+    <t>ZNF165</t>
+  </si>
+  <si>
+    <t>CT53</t>
+  </si>
+  <si>
+    <t>zinc finger protein 165</t>
+  </si>
+  <si>
+    <t>HGNC:2736</t>
+  </si>
+  <si>
+    <t>ENSG00000013573</t>
+  </si>
+  <si>
+    <t>GENE ID:1663</t>
+  </si>
+  <si>
+    <t>DDX11</t>
+  </si>
+  <si>
+    <t>CHLR1</t>
+  </si>
+  <si>
+    <t>DEAD/H-box helicase 11</t>
+  </si>
+  <si>
+    <t>HGNC:13994</t>
+  </si>
+  <si>
+    <t>ENSG00000164256</t>
+  </si>
+  <si>
+    <t>GENE ID:56979</t>
+  </si>
+  <si>
+    <t>PRDM9</t>
+  </si>
+  <si>
+    <t>Meisetz</t>
+  </si>
+  <si>
+    <t>PR/SET domain 9</t>
+  </si>
+  <si>
+    <t>HGNC:1940</t>
+  </si>
+  <si>
+    <t>ENSG00000188419</t>
+  </si>
+  <si>
+    <t>GENE ID:1121</t>
+  </si>
+  <si>
+    <t>CHM</t>
+  </si>
+  <si>
+    <t>HSD-32</t>
+  </si>
+  <si>
+    <t>CHM Rab escort protein</t>
+  </si>
+  <si>
+    <t>HGNC:10115</t>
+  </si>
+  <si>
+    <t>ENSG00000274266</t>
+  </si>
+  <si>
+    <t>GENE ID:6080</t>
+  </si>
+  <si>
+    <t>SNORA73A</t>
+  </si>
+  <si>
+    <t>E1-7</t>
+  </si>
+  <si>
+    <t>small nucleolar RNA, H/ACA box 73A</t>
+  </si>
+  <si>
+    <t>HGNC:1511</t>
+  </si>
+  <si>
+    <t>ENSG00000132906</t>
+  </si>
+  <si>
+    <t>GENE ID:842</t>
+  </si>
+  <si>
+    <t>CASP9</t>
+  </si>
+  <si>
+    <t>MCH6</t>
+  </si>
+  <si>
+    <t>caspase 9</t>
+  </si>
+  <si>
+    <t>HGNC:19881</t>
+  </si>
+  <si>
+    <t>ENSG00000132205</t>
+  </si>
+  <si>
+    <t>GENE ID:84034</t>
+  </si>
+  <si>
+    <t>EMILIN2</t>
+  </si>
+  <si>
+    <t>EMILIN-2</t>
+  </si>
+  <si>
+    <t>elastin microfibril interfacer 2</t>
+  </si>
+  <si>
+    <t>HGNC:2750</t>
+  </si>
+  <si>
+    <t>ENSG00000135829</t>
+  </si>
+  <si>
+    <t>GENE ID:1660</t>
+  </si>
+  <si>
+    <t>DHX9</t>
+  </si>
+  <si>
+    <t>NDH2</t>
+  </si>
+  <si>
+    <t>DExH-box helicase 9</t>
+  </si>
+  <si>
+    <t>HGNC:10478</t>
+  </si>
+  <si>
+    <t>ENSG00000204231</t>
+  </si>
+  <si>
+    <t>GENE ID:6257</t>
+  </si>
+  <si>
+    <t>RXRB</t>
+  </si>
+  <si>
+    <t>DAUDI6</t>
+  </si>
+  <si>
+    <t>retinoid X receptor beta</t>
+  </si>
+  <si>
+    <t>HGNC:12509</t>
+  </si>
+  <si>
+    <t>ENSG00000188021</t>
+  </si>
+  <si>
+    <t>GENE ID:29978</t>
+  </si>
+  <si>
+    <t>UBQLN2</t>
+  </si>
+  <si>
+    <t>Chap1</t>
+  </si>
+  <si>
+    <t>ubiquilin 2</t>
+  </si>
+  <si>
+    <t>HGNC:18133</t>
+  </si>
+  <si>
+    <t>ENSG00000135090</t>
+  </si>
+  <si>
+    <t>GENE ID:51347</t>
+  </si>
+  <si>
+    <t>TAOK3</t>
+  </si>
+  <si>
+    <t>hKFC-A</t>
+  </si>
+  <si>
+    <t>TAO kinase 3</t>
+  </si>
+  <si>
+    <t>HGNC:26435</t>
+  </si>
+  <si>
+    <t>ENSG00000276914, ENSG00000133393</t>
+  </si>
+  <si>
+    <t>GENE ID:123811</t>
+  </si>
+  <si>
+    <t>CEP20</t>
+  </si>
+  <si>
+    <t>FOR20</t>
+  </si>
+  <si>
+    <t>centrosomal protein 20</t>
+  </si>
+  <si>
+    <t>HGNC:28393</t>
+  </si>
+  <si>
+    <t>ENSG00000158792</t>
+  </si>
+  <si>
+    <t>GENE ID:124044</t>
+  </si>
+  <si>
+    <t>SPATA2L</t>
+  </si>
+  <si>
+    <t>tamo</t>
+  </si>
+  <si>
+    <t>spermatogenesis associated 2 like</t>
+  </si>
+  <si>
+    <t>HGNC:21390</t>
+  </si>
+  <si>
+    <t>ENSG00000203877</t>
+  </si>
+  <si>
+    <t>GENE ID:134701</t>
+  </si>
+  <si>
+    <t>RIPPLY2</t>
+  </si>
+  <si>
+    <t>dJ237I15.1</t>
+  </si>
+  <si>
+    <t>ripply transcriptional repressor 2</t>
+  </si>
+  <si>
+    <t>HGNC:54867</t>
+  </si>
+  <si>
+    <t>ENSG00000253712</t>
+  </si>
+  <si>
+    <t>LINC02886</t>
+  </si>
+  <si>
+    <t>RP11-697M17.1</t>
+  </si>
+  <si>
+    <t>long intergenic non-protein coding RNA 2886</t>
+  </si>
+  <si>
+    <t>HGNC:29608</t>
+  </si>
+  <si>
+    <t>ENSG00000147649</t>
+  </si>
+  <si>
+    <t>GENE ID:92140</t>
+  </si>
+  <si>
+    <t>MTDH</t>
+  </si>
+  <si>
+    <t>LYRIC</t>
+  </si>
+  <si>
+    <t>metadherin</t>
+  </si>
+  <si>
+    <t>HGNC:20367</t>
+  </si>
+  <si>
+    <t>ENSG00000073910</t>
+  </si>
+  <si>
+    <t>GENE ID:10129</t>
+  </si>
+  <si>
+    <t>FRY</t>
+  </si>
+  <si>
+    <t>BA37E23.1</t>
+  </si>
+  <si>
+    <t>FRY microtubule binding protein</t>
+  </si>
+  <si>
+    <t>HGNC:24356</t>
+  </si>
+  <si>
+    <t>ENSG00000165682</t>
+  </si>
+  <si>
+    <t>GENE ID:51266</t>
+  </si>
+  <si>
+    <t>CLEC1B</t>
+  </si>
+  <si>
+    <t>1810061I13Rik</t>
+  </si>
+  <si>
+    <t>C-type lectin domain family 1 member B</t>
+  </si>
+  <si>
+    <t>HGNC:11345</t>
+  </si>
+  <si>
+    <t>ENSG00000122707</t>
+  </si>
+  <si>
+    <t>GENE ID:8434</t>
+  </si>
+  <si>
+    <t>RECK</t>
+  </si>
+  <si>
+    <t>hRECK</t>
+  </si>
+  <si>
+    <t>reversion inducing cysteine rich protein with kazal motifs</t>
+  </si>
+  <si>
+    <t>HGNC:50627</t>
+  </si>
+  <si>
+    <t>ENSG00000260887</t>
+  </si>
+  <si>
+    <t>GENE ID:107983961, GENE ID:283854</t>
+  </si>
+  <si>
+    <t>CASC22</t>
+  </si>
+  <si>
+    <t>TCONS_00024290</t>
+  </si>
+  <si>
+    <t>cancer susceptibility 22</t>
+  </si>
+  <si>
+    <t>HGNC:36869</t>
+  </si>
+  <si>
+    <t>ENSG00000219755</t>
+  </si>
+  <si>
+    <t>GENE ID:100131956</t>
+  </si>
+  <si>
+    <t>RPS3P5</t>
+  </si>
+  <si>
+    <t>RPS3_2_726</t>
+  </si>
+  <si>
+    <t>ribosomal protein S3 pseudogene 5</t>
+  </si>
+  <si>
+    <t>HGNC:15985</t>
+  </si>
+  <si>
+    <t>ENSG00000165124</t>
+  </si>
+  <si>
+    <t>GENE ID:79987</t>
+  </si>
+  <si>
+    <t>SVEP1</t>
+  </si>
+  <si>
+    <t>SELOB</t>
+  </si>
+  <si>
+    <t>sushi, von Willebrand factor type A, EGF and pentraxin domain containing 1</t>
+  </si>
+  <si>
+    <t>HGNC:19016</t>
+  </si>
+  <si>
+    <t>ENSG00000166326</t>
+  </si>
+  <si>
+    <t>GENE ID:54765</t>
+  </si>
+  <si>
+    <t>TRIM44</t>
+  </si>
+  <si>
+    <t>HSA249128</t>
+  </si>
+  <si>
+    <t>tripartite motif containing 44</t>
+  </si>
+  <si>
+    <t>HGNC:36798</t>
+  </si>
+  <si>
+    <t>GENE ID:100271022</t>
+  </si>
+  <si>
+    <t>RPL39P11</t>
+  </si>
+  <si>
+    <t>RPL39_3_134</t>
+  </si>
+  <si>
+    <t>ribosomal protein L39 pseudogene 11</t>
+  </si>
+  <si>
+    <t>HGNC:14372</t>
+  </si>
+  <si>
+    <t>ENSG00000142186</t>
+  </si>
+  <si>
+    <t>GENE ID:57410</t>
+  </si>
+  <si>
+    <t>SCYL1</t>
+  </si>
+  <si>
+    <t>HT019</t>
+  </si>
+  <si>
+    <t>SCY1 like pseudokinase 1</t>
+  </si>
+  <si>
+    <t>HGNC:9823</t>
+  </si>
+  <si>
+    <t>ENSG00000185379</t>
+  </si>
+  <si>
+    <t>GENE ID:5892</t>
+  </si>
+  <si>
+    <t>RAD51D</t>
+  </si>
+  <si>
+    <t>HsTRAD</t>
+  </si>
+  <si>
+    <t>RAD51 paralog D</t>
+  </si>
+  <si>
+    <t>HGNC:1555</t>
+  </si>
+  <si>
+    <t>ENSG00000094916</t>
+  </si>
+  <si>
+    <t>GENE ID:23468</t>
+  </si>
+  <si>
+    <t>CBX5</t>
+  </si>
+  <si>
+    <t>HEL25</t>
+  </si>
+  <si>
+    <t>chromobox 5</t>
+  </si>
+  <si>
+    <t>HGNC:9309</t>
+  </si>
+  <si>
+    <t>ENSG00000066027</t>
+  </si>
+  <si>
+    <t>GENE ID:5525</t>
+  </si>
+  <si>
+    <t>PPP2R5A</t>
+  </si>
+  <si>
+    <t>B56ALPHA</t>
+  </si>
+  <si>
+    <t>protein phosphatase 2 regulatory subunit B'alpha</t>
+  </si>
+  <si>
+    <t>HGNC:30290</t>
+  </si>
+  <si>
+    <t>ENSG00000115137</t>
+  </si>
+  <si>
+    <t>GENE ID:51277</t>
+  </si>
+  <si>
+    <t>DNAJC27</t>
+  </si>
+  <si>
+    <t>RABJS</t>
+  </si>
+  <si>
+    <t>DnaJ heat shock protein family (Hsp40) member C27</t>
+  </si>
+  <si>
+    <t>HGNC:24748</t>
+  </si>
+  <si>
+    <t>ENSG00000175984</t>
+  </si>
+  <si>
+    <t>GENE ID:163259</t>
+  </si>
+  <si>
+    <t>DENND2C</t>
+  </si>
+  <si>
+    <t>dJ1156J9.1</t>
+  </si>
+  <si>
+    <t>DENN domain containing 2C</t>
+  </si>
+  <si>
+    <t>HGNC:18001</t>
+  </si>
+  <si>
+    <t>ENSG00000130204</t>
+  </si>
+  <si>
+    <t>GENE ID:10452</t>
+  </si>
+  <si>
+    <t>TOMM40</t>
+  </si>
+  <si>
+    <t>PEREC1</t>
+  </si>
+  <si>
+    <t>translocase of outer mitochondrial membrane 40</t>
+  </si>
+  <si>
+    <t>HGNC:18475</t>
+  </si>
+  <si>
+    <t>ENSG00000188706</t>
+  </si>
+  <si>
+    <t>GENE ID:51114</t>
+  </si>
+  <si>
+    <t>ZDHHC9</t>
+  </si>
+  <si>
+    <t>ZNF379</t>
+  </si>
+  <si>
+    <t>zDHHC palmitoyltransferase 9</t>
+  </si>
+  <si>
+    <t>HGNC:17851</t>
+  </si>
+  <si>
+    <t>ENSG00000076043</t>
+  </si>
+  <si>
+    <t>GENE ID:25996</t>
+  </si>
+  <si>
+    <t>REXO2</t>
+  </si>
+  <si>
+    <t>RFN</t>
+  </si>
+  <si>
+    <t>RNA exonuclease 2</t>
+  </si>
+  <si>
+    <t>HGNC:9564</t>
+  </si>
+  <si>
+    <t>ENSG00000163636</t>
+  </si>
+  <si>
+    <t>GENE ID:9861</t>
+  </si>
+  <si>
+    <t>PSMD6</t>
+  </si>
+  <si>
+    <t>p44S10</t>
+  </si>
+  <si>
+    <t>proteasome 26S subunit, non-ATPase 6</t>
+  </si>
+  <si>
+    <t>HGNC:16412</t>
+  </si>
+  <si>
+    <t>ENSG00000091106</t>
+  </si>
+  <si>
+    <t>GENE ID:58484</t>
+  </si>
+  <si>
+    <t>NLRC4</t>
+  </si>
+  <si>
+    <t>CLANA</t>
+  </si>
+  <si>
+    <t>NLR family CARD domain containing 4</t>
+  </si>
+  <si>
+    <t>HGNC:6903</t>
+  </si>
+  <si>
+    <t>ENSG00000151224</t>
+  </si>
+  <si>
+    <t>GENE ID:4143</t>
+  </si>
+  <si>
+    <t>MAT1A</t>
+  </si>
+  <si>
+    <t>SAMS1</t>
+  </si>
+  <si>
+    <t>methionine adenosyltransferase 1A</t>
+  </si>
+  <si>
+    <t>HGNC:23068</t>
+  </si>
+  <si>
+    <t>ENSG00000196459</t>
+  </si>
+  <si>
+    <t>GENE ID:6399</t>
+  </si>
+  <si>
+    <t>TRAPPC2</t>
+  </si>
+  <si>
+    <t>ZNF547L</t>
+  </si>
+  <si>
+    <t>trafficking protein particle complex subunit 2</t>
+  </si>
+  <si>
+    <t>HGNC:28669</t>
+  </si>
+  <si>
+    <t>ENSG00000198870</t>
+  </si>
+  <si>
+    <t>GENE ID:169436</t>
+  </si>
+  <si>
+    <t>STKLD1</t>
+  </si>
+  <si>
+    <t>Sk521</t>
+  </si>
+  <si>
+    <t>serine/threonine kinase like domain containing 1</t>
+  </si>
+  <si>
+    <t>HGNC:30757</t>
+  </si>
+  <si>
+    <t>ENSG00000145087</t>
+  </si>
+  <si>
+    <t>GENE ID:9515</t>
+  </si>
+  <si>
+    <t>STXBP5L</t>
+  </si>
+  <si>
+    <t>TOMOSYN-2</t>
+  </si>
+  <si>
+    <t>syntaxin binding protein 5L</t>
+  </si>
+  <si>
+    <t>HGNC:33719</t>
+  </si>
+  <si>
+    <t>ENSG00000188807</t>
+  </si>
+  <si>
+    <t>GENE ID:199953</t>
+  </si>
+  <si>
+    <t>TMEM201</t>
+  </si>
+  <si>
+    <t>RP13-15M17.2</t>
+  </si>
+  <si>
+    <t>transmembrane protein 201</t>
+  </si>
+  <si>
+    <t>HGNC:4606</t>
+  </si>
+  <si>
+    <t>ENSG00000167004</t>
+  </si>
+  <si>
+    <t>GENE ID:2923</t>
+  </si>
+  <si>
+    <t>PDIA3</t>
+  </si>
+  <si>
+    <t>HEL-S-93n</t>
+  </si>
+  <si>
+    <t>protein disulfide isomerase family A member 3</t>
+  </si>
+  <si>
+    <t>HGNC:16641</t>
+  </si>
+  <si>
+    <t>ENSG00000176358</t>
+  </si>
+  <si>
+    <t>GENE ID:255061</t>
+  </si>
+  <si>
+    <t>TAC4</t>
+  </si>
+  <si>
+    <t>HK1</t>
+  </si>
+  <si>
+    <t>tachykinin precursor 4</t>
+  </si>
+  <si>
+    <t>HGNC:330</t>
+  </si>
+  <si>
+    <t>ENSG00000159723</t>
+  </si>
+  <si>
+    <t>GENE ID:181</t>
+  </si>
+  <si>
+    <t>AGRP</t>
+  </si>
+  <si>
+    <t>ASIP2</t>
+  </si>
+  <si>
+    <t>agouti related neuropeptide</t>
+  </si>
+  <si>
+    <t>HGNC:56665</t>
+  </si>
+  <si>
+    <t>ENSG00000231412</t>
+  </si>
+  <si>
+    <t>GENE ID:128193286</t>
+  </si>
+  <si>
+    <t>LINC03078</t>
+  </si>
+  <si>
+    <t>AC005392.2</t>
+  </si>
+  <si>
+    <t>long intergenic non-protein coding RNA 3078</t>
+  </si>
+  <si>
+    <t>HGNC:3537</t>
+  </si>
+  <si>
+    <t>ENSG00000181104</t>
+  </si>
+  <si>
+    <t>GENE ID:2149</t>
+  </si>
+  <si>
+    <t>F2R</t>
+  </si>
+  <si>
+    <t>PAR1</t>
+  </si>
+  <si>
+    <t>coagulation factor II thrombin receptor</t>
+  </si>
+  <si>
+    <t>HGNC:8406</t>
+  </si>
+  <si>
+    <t>ENSG00000226537</t>
+  </si>
+  <si>
+    <t>GENE ID:26640</t>
+  </si>
+  <si>
+    <t>OR7E33P</t>
+  </si>
+  <si>
+    <t>hg688</t>
+  </si>
+  <si>
+    <t>olfactory receptor family 7 subfamily E member 33 pseudogene</t>
+  </si>
+  <si>
+    <t>HGNC:9566</t>
+  </si>
+  <si>
+    <t>ENSG00000099341</t>
+  </si>
+  <si>
+    <t>GENE ID:5714</t>
+  </si>
+  <si>
+    <t>PSMD8</t>
+  </si>
+  <si>
+    <t>S14</t>
+  </si>
+  <si>
+    <t>proteasome 26S subunit, non-ATPase 8</t>
+  </si>
+  <si>
+    <t>HGNC:12195</t>
+  </si>
+  <si>
+    <t>ENSG00000226660, ENSG00000282568</t>
+  </si>
+  <si>
+    <t>GENE ID:28620</t>
+  </si>
+  <si>
+    <t>TRBV2</t>
+  </si>
+  <si>
+    <t>TCRBV22S1A2N1T</t>
+  </si>
+  <si>
+    <t>T cell receptor beta variable 2</t>
+  </si>
+  <si>
+    <t>HGNC:5951</t>
+  </si>
+  <si>
+    <t>ENSG00000182985</t>
+  </si>
+  <si>
+    <t>GENE ID:23705</t>
+  </si>
+  <si>
+    <t>CADM1</t>
+  </si>
+  <si>
+    <t>NECL-2</t>
+  </si>
+  <si>
+    <t>cell adhesion molecule 1</t>
+  </si>
+  <si>
+    <t>HGNC:4872</t>
+  </si>
+  <si>
+    <t>ENSG00000230267</t>
+  </si>
+  <si>
+    <t>GENE ID:100289574</t>
+  </si>
+  <si>
+    <t>HERC2P4</t>
+  </si>
+  <si>
+    <t>D16F37S5</t>
+  </si>
+  <si>
+    <t>HERC2 pseudogene 4</t>
+  </si>
+  <si>
+    <t>HGNC:36733</t>
+  </si>
+  <si>
+    <t>ENSG00000236264</t>
+  </si>
+  <si>
+    <t>GENE ID:653147</t>
+  </si>
+  <si>
+    <t>RPL26P30</t>
+  </si>
+  <si>
+    <t>RPL26_10_1113</t>
+  </si>
+  <si>
+    <t>ribosomal protein L26 pseudogene 30</t>
+  </si>
+  <si>
+    <t>HGNC:4516</t>
+  </si>
+  <si>
+    <t>ENSG00000173698</t>
+  </si>
+  <si>
+    <t>GENE ID:10149</t>
+  </si>
+  <si>
+    <t>ADGRG2</t>
+  </si>
+  <si>
+    <t>HE6</t>
+  </si>
+  <si>
+    <t>adhesion G protein-coupled receptor G2</t>
+  </si>
+  <si>
+    <t>HGNC:3167</t>
+  </si>
+  <si>
+    <t>ENSG00000213694</t>
+  </si>
+  <si>
+    <t>GENE ID:1903</t>
+  </si>
+  <si>
+    <t>S1PR3</t>
+  </si>
+  <si>
+    <t>EDG-3</t>
+  </si>
+  <si>
+    <t>sphingosine-1-phosphate receptor 3</t>
+  </si>
+  <si>
+    <t>HGNC:14558</t>
+  </si>
+  <si>
+    <t>ENSG00000172243</t>
+  </si>
+  <si>
+    <t>GENE ID:64581</t>
+  </si>
+  <si>
+    <t>CLEC7A</t>
+  </si>
+  <si>
+    <t>DECTIN1</t>
+  </si>
+  <si>
+    <t>C-type lectin domain containing 7A</t>
+  </si>
+  <si>
+    <t>HGNC:11958</t>
+  </si>
+  <si>
+    <t>ENSG00000183495</t>
+  </si>
+  <si>
+    <t>GENE ID:57634</t>
+  </si>
+  <si>
+    <t>EP400</t>
+  </si>
+  <si>
+    <t>CAGH32</t>
+  </si>
+  <si>
+    <t>E1A binding protein p400</t>
+  </si>
+  <si>
+    <t>HGNC:5409</t>
+  </si>
+  <si>
+    <t>ENSG00000119922</t>
+  </si>
+  <si>
+    <t>GENE ID:3433</t>
+  </si>
+  <si>
+    <t>IFIT2</t>
+  </si>
+  <si>
+    <t>cig42</t>
+  </si>
+  <si>
+    <t>interferon induced protein with tetratricopeptide repeats 2</t>
+  </si>
+  <si>
+    <t>HGNC:20182</t>
+  </si>
+  <si>
+    <t>ENSG00000029364</t>
+  </si>
+  <si>
+    <t>GENE ID:55334</t>
+  </si>
+  <si>
+    <t>SLC39A9</t>
+  </si>
+  <si>
+    <t>ZIP-9</t>
+  </si>
+  <si>
+    <t>solute carrier family 39 member 9</t>
+  </si>
+  <si>
+    <t>HGNC:32419</t>
+  </si>
+  <si>
+    <t>ENSG00000183054</t>
+  </si>
+  <si>
+    <t>GENE ID:729540</t>
+  </si>
+  <si>
+    <t>RGPD6</t>
+  </si>
+  <si>
+    <t>RanBP2L2</t>
+  </si>
+  <si>
+    <t>RANBP2 like and GRIP domain containing 6</t>
+  </si>
+  <si>
+    <t>HGNC:48</t>
+  </si>
+  <si>
+    <t>ENSG00000131269</t>
+  </si>
+  <si>
+    <t>GENE ID:22</t>
+  </si>
+  <si>
+    <t>ABCB7</t>
+  </si>
+  <si>
+    <t>Atm1p</t>
+  </si>
+  <si>
+    <t>ATP binding cassette subfamily B member 7</t>
+  </si>
+  <si>
+    <t>HGNC:36791</t>
+  </si>
+  <si>
+    <t>GENE ID:100271646</t>
+  </si>
+  <si>
+    <t>RPL36AP43</t>
+  </si>
+  <si>
+    <t>RPL36A_21_1460</t>
+  </si>
+  <si>
+    <t>ribosomal protein L36a pseudogene 43</t>
+  </si>
+  <si>
+    <t>HGNC:7505</t>
+  </si>
+  <si>
+    <t>ENSG00000236675</t>
+  </si>
+  <si>
+    <t>GENE ID:4581</t>
+  </si>
+  <si>
+    <t>MTX1LP</t>
+  </si>
+  <si>
+    <t>psMTX</t>
+  </si>
+  <si>
+    <t>metaxin 1 like, pseudogene</t>
+  </si>
+  <si>
+    <t>HGNC:24845</t>
+  </si>
+  <si>
+    <t>ENSG00000135631</t>
+  </si>
+  <si>
+    <t>GENE ID:26056</t>
+  </si>
+  <si>
+    <t>RAB11FIP5</t>
+  </si>
+  <si>
+    <t>pp75</t>
+  </si>
+  <si>
+    <t>RAB11 family interacting protein 5</t>
+  </si>
+  <si>
+    <t>HGNC:10924</t>
+  </si>
+  <si>
+    <t>ENSG00000141526</t>
+  </si>
+  <si>
+    <t>GENE ID:9123</t>
+  </si>
+  <si>
+    <t>SLC16A3</t>
+  </si>
+  <si>
+    <t>MCT3</t>
+  </si>
+  <si>
+    <t>solute carrier family 16 member 3</t>
+  </si>
+  <si>
+    <t>HGNC:16091</t>
+  </si>
+  <si>
+    <t>ENSG00000154930</t>
+  </si>
+  <si>
+    <t>GENE ID:84532</t>
+  </si>
+  <si>
+    <t>ACSS1</t>
+  </si>
+  <si>
+    <t>ACECS2L</t>
+  </si>
+  <si>
+    <t>acyl-CoA synthetase short chain family member 1</t>
+  </si>
+  <si>
+    <t>HGNC:30422</t>
+  </si>
+  <si>
+    <t>ENSG00000138771</t>
+  </si>
+  <si>
+    <t>GENE ID:57619</t>
+  </si>
+  <si>
+    <t>SHROOM3</t>
+  </si>
+  <si>
+    <t>APXL3</t>
+  </si>
+  <si>
+    <t>shroom family member 3</t>
+  </si>
+  <si>
+    <t>HGNC:28789</t>
+  </si>
+  <si>
+    <t>ENSG00000133872</t>
+  </si>
+  <si>
+    <t>GENE ID:51669</t>
+  </si>
+  <si>
+    <t>SARAF</t>
+  </si>
+  <si>
+    <t>HSPC035</t>
+  </si>
+  <si>
+    <t>store-operated calcium entry associated regulatory factor</t>
+  </si>
+  <si>
+    <t>HGNC:978</t>
+  </si>
+  <si>
+    <t>ENSG00000107949</t>
+  </si>
+  <si>
+    <t>GENE ID:56647</t>
+  </si>
+  <si>
+    <t>BCCIP</t>
+  </si>
+  <si>
+    <t>BCCIPalpha</t>
+  </si>
+  <si>
+    <t>BRCA2 and CDKN1A interacting protein</t>
+  </si>
+  <si>
+    <t>HGNC:16487</t>
+  </si>
+  <si>
+    <t>ENSG00000184060</t>
+  </si>
+  <si>
+    <t>GENE ID:55803</t>
+  </si>
+  <si>
+    <t>ADAP2</t>
+  </si>
+  <si>
+    <t>HSA272195</t>
+  </si>
+  <si>
+    <t>ArfGAP with dual PH domains 2</t>
   </si>
 </sst>
 </file>
@@ -567,8 +1818,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:I31" totalsRowShown="0">
-  <autoFilter ref="A1:I31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:I101" totalsRowShown="0">
+  <autoFilter ref="A1:I101"/>
   <tableColumns count="9">
     <tableColumn id="1" name="HGNC_ID" dataDxfId="0"/>
     <tableColumn id="2" name="ENSG_ID" dataDxfId="0"/>
@@ -869,7 +2120,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I31"/>
+  <dimension ref="A1:I101"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1721,6 +2972,1896 @@
       </c>
       <c r="I31" s="1" t="s">
         <v>166</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="D32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H32" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="D33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="H33" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" s="1" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H34" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="D35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="H35" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" s="1" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="H36" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="D37" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H37" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="H38" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="D39" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="H39" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I39" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D40" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="H40" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="H41" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I41" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="H42" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I42" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="D43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H43" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I43" s="1" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D44" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="H44" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I44" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="D45" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="H45" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I45" s="1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D46" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H46" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="D47" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H47" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D48" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="H48" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="D49" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H49" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="D50" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H50" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="D51" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E51" s="1"/>
+      <c r="F51" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H51" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I51" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="D52" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E52" s="1"/>
+      <c r="F52" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="H52" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I52" s="1" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="D53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="H53" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I53" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D54" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="H54" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I54" s="1" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="H55" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="D56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="H56" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D57" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="H57" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="D58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="H58" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="D59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="H59" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" s="1" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D60" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="H60" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="D61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="H61" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" s="1" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="D62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="H62" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D63" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="H63" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="D64" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E64" s="1"/>
+      <c r="F64" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="H64" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="D65" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="H65" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="D66" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E66" s="1"/>
+      <c r="F66" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="H66" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D67" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E67" s="1"/>
+      <c r="F67" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="H67" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D68" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E68" s="1"/>
+      <c r="F68" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="H68" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="1" t="s">
+        <v>387</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="D69" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E69" s="1"/>
+      <c r="F69" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="H69" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="D70" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="H70" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" s="1" t="s">
+        <v>399</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>400</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="D71" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E71" s="1"/>
+      <c r="F71" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="H71" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>406</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="D72" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E72" s="1"/>
+      <c r="F72" s="1" t="s">
+        <v>408</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="H72" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" s="1" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="D73" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="H73" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" s="1" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9">
+      <c r="A74" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="D74" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E74" s="1"/>
+      <c r="F74" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="H74" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="D75" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" s="1"/>
+      <c r="F75" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="H75" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>430</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="D76" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1" t="s">
+        <v>432</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="H76" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" s="1" t="s">
+        <v>435</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>437</v>
+      </c>
+      <c r="D77" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E77" s="1"/>
+      <c r="F77" s="1" t="s">
+        <v>438</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>439</v>
+      </c>
+      <c r="H77" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" s="1" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="D78" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E78" s="1"/>
+      <c r="F78" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="H78" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" s="1" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" s="1" t="s">
+        <v>447</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="D79" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="H79" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" s="1" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>454</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="D80" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E80" s="1"/>
+      <c r="F80" s="1" t="s">
+        <v>456</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="H80" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" s="1" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>460</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="D81" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E81" s="1"/>
+      <c r="F81" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="H81" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" s="1" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" s="1" t="s">
+        <v>465</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>467</v>
+      </c>
+      <c r="D82" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E82" s="1"/>
+      <c r="F82" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="H82" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" s="1" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" s="1" t="s">
+        <v>471</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="D83" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E83" s="1"/>
+      <c r="F83" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="H83" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="D84" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E84" s="1"/>
+      <c r="F84" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>481</v>
+      </c>
+      <c r="H84" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" s="1" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="D85" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E85" s="1"/>
+      <c r="F85" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="H85" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" s="1" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" s="1" t="s">
+        <v>489</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="D86" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="H86" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" s="1" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" s="1" t="s">
+        <v>495</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>497</v>
+      </c>
+      <c r="D87" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1" t="s">
+        <v>498</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>499</v>
+      </c>
+      <c r="H87" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" s="1" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9">
+      <c r="A88" s="1" t="s">
+        <v>501</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>502</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="D88" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E88" s="1"/>
+      <c r="F88" s="1" t="s">
+        <v>504</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="H88" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" s="1" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>508</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>509</v>
+      </c>
+      <c r="D89" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E89" s="1"/>
+      <c r="F89" s="1" t="s">
+        <v>510</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>511</v>
+      </c>
+      <c r="H89" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" s="1" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9">
+      <c r="A90" s="1" t="s">
+        <v>513</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>515</v>
+      </c>
+      <c r="D90" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E90" s="1"/>
+      <c r="F90" s="1" t="s">
+        <v>516</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>517</v>
+      </c>
+      <c r="H90" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" s="1" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9">
+      <c r="A91" s="1" t="s">
+        <v>519</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>520</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="D91" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E91" s="1"/>
+      <c r="F91" s="1" t="s">
+        <v>522</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>523</v>
+      </c>
+      <c r="H91" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9">
+      <c r="A92" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="D92" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E92" s="1"/>
+      <c r="F92" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="H92" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9">
+      <c r="A93" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="D93" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E93" s="1"/>
+      <c r="F93" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="H93" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" s="1" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9">
+      <c r="A94" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="D94" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E94" s="1"/>
+      <c r="F94" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="H94" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9">
+      <c r="A95" s="1" t="s">
+        <v>542</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>543</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="D95" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E95" s="1"/>
+      <c r="F95" s="1" t="s">
+        <v>545</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="H95" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9">
+      <c r="A96" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>550</v>
+      </c>
+      <c r="D96" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E96" s="1"/>
+      <c r="F96" s="1" t="s">
+        <v>551</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="H96" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9">
+      <c r="A97" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>555</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="D97" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E97" s="1"/>
+      <c r="F97" s="1" t="s">
+        <v>557</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="H97" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9">
+      <c r="A98" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>561</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>562</v>
+      </c>
+      <c r="D98" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E98" s="1"/>
+      <c r="F98" s="1" t="s">
+        <v>563</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>564</v>
+      </c>
+      <c r="H98" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9">
+      <c r="A99" s="1" t="s">
+        <v>566</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>567</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>568</v>
+      </c>
+      <c r="D99" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E99" s="1"/>
+      <c r="F99" s="1" t="s">
+        <v>569</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>570</v>
+      </c>
+      <c r="H99" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9">
+      <c r="A100" s="1" t="s">
+        <v>572</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>573</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>574</v>
+      </c>
+      <c r="D100" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E100" s="1"/>
+      <c r="F100" s="1" t="s">
+        <v>575</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>576</v>
+      </c>
+      <c r="H100" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9">
+      <c r="A101" s="1" t="s">
+        <v>578</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>579</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>580</v>
+      </c>
+      <c r="D101" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="E101" s="1"/>
+      <c r="F101" s="1" t="s">
+        <v>581</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>582</v>
+      </c>
+      <c r="H101" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>583</v>
       </c>
     </row>
   </sheetData>

</xml_diff>